<commit_message>
Update removing test tab sync
</commit_message>
<xml_diff>
--- a/data/Master AHRI (3).xlsx
+++ b/data/Master AHRI (3).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\konis\AHRI Estimator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA703703-639E-4C86-8A83-B0E7792B17FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC296083-B462-43A6-AD63-BC7A584B08E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2-Ton Gas" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,6 @@
     <sheet name="5-Ton Gas" sheetId="6" r:id="rId16"/>
     <sheet name="5-Ton HP" sheetId="17" r:id="rId17"/>
     <sheet name="5-Ton Gas SC" sheetId="18" r:id="rId18"/>
-    <sheet name="TEST" sheetId="19" r:id="rId19"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -1282,109 +1281,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60B01F1D-2266-4B3E-BD77-EDC4B18EA26B}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:A18"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1">
-        <v>214858034</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>215378866</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>217655941</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>215489155</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>217655941</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>215213843</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>215381153</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>215657375</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>215429185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>217989106</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>214857992</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>215378838</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>215865227</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>215445893</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>217109134</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>214860184</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>215213862</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>214860141</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{852330AB-2968-4791-AD8E-74D1CF5BEE16}">
   <sheetPr>

</xml_diff>

<commit_message>
Updated 2-ton ahri units
</commit_message>
<xml_diff>
--- a/data/Master AHRI (3).xlsx
+++ b/data/Master AHRI (3).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\konis\AHRI Estimator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC296083-B462-43A6-AD63-BC7A584B08E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D94806-2E10-4560-A8F1-70E2C4DFCDD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2-Ton Gas" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -71,18 +71,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -96,13 +84,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -321,7 +307,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
@@ -349,93 +335,13 @@
         <v>216613778</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>215213838</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>215381150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>215657370</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>215429181</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>216699843</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>214858529</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>215377921</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>215865341</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>215445888</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>217178426</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="4">
-        <v>215214628</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="4">
-        <v>215213871</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="4">
-        <v>215214929</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="5">
-        <v>215359084</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="5">
-        <v>215828157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="5">
-        <v>216375597</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22">
+    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>218350555</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23">
+    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>218350701</v>
       </c>
     </row>
@@ -1286,122 +1192,32 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="3">
-        <v>214858688</v>
+        <v>215213838</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
-        <v>215377941</v>
+        <v>215381150</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
-        <v>216613778</v>
+        <v>215657370</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>215488983</v>
+        <v>215429181</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
-        <v>216613778</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>215213838</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>215381150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>215657370</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>215429181</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
         <v>216699843</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>214858529</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>215377921</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>215865341</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>215445888</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>217178426</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="4">
-        <v>215214628</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="4">
-        <v>215213871</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="4">
-        <v>215214929</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="5">
-        <v>215359084</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="5">
-        <v>215828157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="5">
-        <v>216375597</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>218350555</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>218350701</v>
       </c>
     </row>
   </sheetData>
@@ -1414,122 +1230,32 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="3">
-        <v>214858688</v>
+        <v>214858529</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
-        <v>215377941</v>
+        <v>215377921</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
-        <v>216613778</v>
+        <v>215865341</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>215488983</v>
+        <v>215445888</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
-        <v>216613778</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>215213838</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>215381150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>215657370</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>215429181</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>216699843</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>214858529</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>215377921</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>215865341</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>215445888</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
         <v>217178426</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="4">
-        <v>215214628</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="4">
-        <v>215213871</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="4">
-        <v>215214929</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="5">
-        <v>215359084</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="5">
-        <v>215828157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="5">
-        <v>216375597</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>218350555</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>218350701</v>
       </c>
     </row>
   </sheetData>

</xml_diff>